<commit_message>
add RHB Bank Format Excel
</commit_message>
<xml_diff>
--- a/assets/payroll_export_template.xlsx
+++ b/assets/payroll_export_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\hasani_payroll\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D769A080-2A28-48D4-8EEF-09D10659460C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5F02D5-04A5-4513-A7F2-17BD68EF986D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{BB4F4676-B1CA-48B0-BA5A-E4611AFDE364}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>PENYATA GAJI</t>
   </si>
@@ -135,9 +135,6 @@
   </si>
   <si>
     <t>JUMLAH BERSIH</t>
-  </si>
-  <si>
-    <t>TOTAL AMOUNT</t>
   </si>
   <si>
     <t>Anwar</t>
@@ -762,6 +759,15 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="43" fontId="25" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
@@ -792,15 +798,6 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="25" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -2213,28 +2210,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
-      <c r="O1" s="78"/>
-      <c r="P1" s="78"/>
-      <c r="Q1" s="78"/>
-      <c r="R1" s="78"/>
-      <c r="S1" s="78"/>
-      <c r="T1" s="78"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="81"/>
+      <c r="G1" s="81"/>
+      <c r="H1" s="81"/>
+      <c r="I1" s="82"/>
+      <c r="J1" s="81"/>
+      <c r="K1" s="81"/>
+      <c r="L1" s="81"/>
+      <c r="M1" s="81"/>
+      <c r="N1" s="81"/>
+      <c r="O1" s="81"/>
+      <c r="P1" s="81"/>
+      <c r="Q1" s="81"/>
+      <c r="R1" s="81"/>
+      <c r="S1" s="81"/>
+      <c r="T1" s="81"/>
     </row>
     <row r="2" spans="1:24" ht="28.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="2"/>
@@ -2248,41 +2245,41 @@
       <c r="I2" s="3"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="80" t="s">
+      <c r="L2" s="83" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="80"/>
-      <c r="N2" s="80"/>
-      <c r="O2" s="80"/>
-      <c r="P2" s="80"/>
-      <c r="Q2" s="80"/>
+      <c r="M2" s="83"/>
+      <c r="N2" s="83"/>
+      <c r="O2" s="83"/>
+      <c r="P2" s="83"/>
+      <c r="Q2" s="83"/>
       <c r="R2" s="2"/>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
     </row>
     <row r="3" spans="1:24" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="81">
+      <c r="A3" s="84">
         <v>46204</v>
       </c>
-      <c r="B3" s="81"/>
-      <c r="C3" s="81"/>
-      <c r="D3" s="81"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="81"/>
-      <c r="G3" s="81"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="81"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="81"/>
-      <c r="L3" s="81"/>
-      <c r="M3" s="81"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="81"/>
-      <c r="P3" s="81"/>
-      <c r="Q3" s="81"/>
-      <c r="R3" s="81"/>
-      <c r="S3" s="81"/>
-      <c r="T3" s="81"/>
+      <c r="B3" s="84"/>
+      <c r="C3" s="84"/>
+      <c r="D3" s="84"/>
+      <c r="E3" s="84"/>
+      <c r="F3" s="84"/>
+      <c r="G3" s="84"/>
+      <c r="H3" s="84"/>
+      <c r="I3" s="84"/>
+      <c r="J3" s="84"/>
+      <c r="K3" s="84"/>
+      <c r="L3" s="84"/>
+      <c r="M3" s="84"/>
+      <c r="N3" s="84"/>
+      <c r="O3" s="84"/>
+      <c r="P3" s="84"/>
+      <c r="Q3" s="84"/>
+      <c r="R3" s="84"/>
+      <c r="S3" s="84"/>
+      <c r="T3" s="84"/>
     </row>
     <row r="4" spans="1:24" s="10" customFormat="1" ht="50.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -3586,14 +3583,12 @@
       <c r="W52" s="1"/>
     </row>
     <row r="53" spans="1:23" ht="26.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="82" t="s">
-        <v>22</v>
-      </c>
-      <c r="B53" s="83"/>
-      <c r="C53" s="83"/>
-      <c r="D53" s="83"/>
-      <c r="E53" s="83"/>
-      <c r="F53" s="83"/>
+      <c r="A53" s="85"/>
+      <c r="B53" s="86"/>
+      <c r="C53" s="86"/>
+      <c r="D53" s="86"/>
+      <c r="E53" s="86"/>
+      <c r="F53" s="86"/>
       <c r="G53" s="57"/>
       <c r="H53" s="58">
         <f t="shared" ref="H53:T53" si="0">SUM(H5:H52)</f>
@@ -3670,10 +3665,10 @@
     <row r="55" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="60"/>
       <c r="B55" s="60"/>
-      <c r="C55" s="84" t="s">
-        <v>23</v>
-      </c>
-      <c r="D55" s="84"/>
+      <c r="C55" s="87" t="s">
+        <v>22</v>
+      </c>
+      <c r="D55" s="87"/>
       <c r="F55" s="64"/>
       <c r="G55" s="64"/>
       <c r="H55" s="65"/>
@@ -3692,11 +3687,11 @@
     <row r="56" spans="1:23" ht="21.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A56" s="60"/>
       <c r="B56" s="60"/>
-      <c r="C56" s="85"/>
-      <c r="D56" s="85"/>
+      <c r="C56" s="88"/>
+      <c r="D56" s="88"/>
       <c r="F56" s="69"/>
-      <c r="G56" s="86"/>
-      <c r="H56" s="86"/>
+      <c r="G56" s="89"/>
+      <c r="H56" s="89"/>
       <c r="I56" s="69"/>
       <c r="J56" s="69"/>
       <c r="K56" s="69"/>
@@ -3713,14 +3708,14 @@
     <row r="57" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="60"/>
       <c r="B57" s="60"/>
-      <c r="C57" s="89" t="s">
+      <c r="C57" s="80" t="s">
+        <v>23</v>
+      </c>
+      <c r="D57" s="80"/>
+      <c r="G57" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="D57" s="89"/>
-      <c r="G57" s="89" t="s">
-        <v>25</v>
-      </c>
-      <c r="H57" s="89"/>
+      <c r="H57" s="80"/>
       <c r="I57" s="71"/>
       <c r="J57" s="71"/>
       <c r="K57" s="71"/>
@@ -3741,10 +3736,10 @@
       <c r="G58" s="73"/>
       <c r="H58" s="73"/>
       <c r="I58" s="73"/>
-      <c r="J58" s="87"/>
-      <c r="K58" s="87"/>
-      <c r="L58" s="87"/>
-      <c r="M58" s="88"/>
+      <c r="J58" s="78"/>
+      <c r="K58" s="78"/>
+      <c r="L58" s="78"/>
+      <c r="M58" s="79"/>
       <c r="N58" s="22"/>
       <c r="O58" s="22"/>
       <c r="P58" s="22"/>
@@ -3755,10 +3750,10 @@
     </row>
     <row r="59" spans="1:23" ht="18" x14ac:dyDescent="0.25">
       <c r="F59" s="74"/>
-      <c r="J59" s="87"/>
-      <c r="K59" s="87"/>
-      <c r="L59" s="87"/>
-      <c r="M59" s="88"/>
+      <c r="J59" s="78"/>
+      <c r="K59" s="78"/>
+      <c r="L59" s="78"/>
+      <c r="M59" s="79"/>
       <c r="N59" s="22"/>
       <c r="O59" s="22"/>
       <c r="P59" s="22"/>

</xml_diff>